<commit_message>
Release 0.12.0 evaluation analytics
</commit_message>
<xml_diff>
--- a/data/candidates.xlsx
+++ b/data/candidates.xlsx
@@ -600,11 +600,11 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-06-14T16:30:26.381684</t>
+          <t>2026-06-16T15:21:53.406305</t>
         </is>
       </c>
     </row>

</xml_diff>